<commit_message>
changement horaire pour perte de jira
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/support/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C754A1-29F9-8146-ABD6-14446F1140B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C65A8A18-CE0B-6445-8BDC-E4DC342A8525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="27240" windowHeight="16440" activeTab="1" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="56">
   <si>
     <t>Date</t>
   </si>
@@ -270,14 +270,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -647,7 +646,7 @@
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>54</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -923,10 +922,10 @@
         <v>18</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -939,11 +938,11 @@
       <c r="C20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E20" t="s">
-        <v>3</v>
+      <c r="D20" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -956,11 +955,11 @@
       <c r="C21" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>3</v>
+      <c r="D21" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -973,11 +972,11 @@
       <c r="C22" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>3</v>
+      <c r="D22" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -990,10 +989,10 @@
       <c r="C23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" t="s">
         <v>16</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1007,11 +1006,11 @@
       <c r="C24" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>4</v>
+      <c r="D24" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -1021,12 +1020,14 @@
       <c r="B25">
         <v>24</v>
       </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>18</v>
+      <c r="C25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -1039,11 +1040,11 @@
       <c r="C26" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D26" t="s">
-        <v>16</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>18</v>
+      <c r="D26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -1056,11 +1057,11 @@
       <c r="C27" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>18</v>
+      <c r="D27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1173,7 +1174,7 @@
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="6">
         <v>46038.552083333336</v>
       </c>
       <c r="D2" s="2" t="str">
@@ -1196,7 +1197,7 @@
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="6">
         <v>46041.635416666664</v>
       </c>
       <c r="D3" s="2" t="str">
@@ -1219,7 +1220,7 @@
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>46045.552083333336</v>
       </c>
       <c r="D4" s="2" t="str">
@@ -1242,7 +1243,7 @@
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>46048.635416666664</v>
       </c>
       <c r="D5" s="2" t="str">
@@ -1265,7 +1266,7 @@
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>46052.552083333336</v>
       </c>
       <c r="D6" s="2" t="str">
@@ -1288,7 +1289,7 @@
       <c r="B7">
         <v>6</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>46055.635416666664</v>
       </c>
       <c r="D7" s="2" t="str">
@@ -1311,7 +1312,7 @@
       <c r="B8">
         <v>7</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <v>46059.552083333336</v>
       </c>
       <c r="D8" s="2" t="str">
@@ -1334,7 +1335,7 @@
       <c r="B9">
         <v>8</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <v>46062.635416666664</v>
       </c>
       <c r="D9" s="2" t="str">
@@ -1357,7 +1358,7 @@
       <c r="B10">
         <v>9</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <v>46066.552083333336</v>
       </c>
       <c r="D10" s="2" t="str">
@@ -1380,7 +1381,7 @@
       <c r="B11">
         <v>10</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <v>46069.635416666664</v>
       </c>
       <c r="D11" s="2" t="str">
@@ -1403,7 +1404,7 @@
       <c r="B12">
         <v>11</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="6">
         <v>46073.552083333336</v>
       </c>
       <c r="D12" s="2" t="str">
@@ -1426,7 +1427,7 @@
       <c r="B13">
         <v>12</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="6">
         <v>46076.635416666664</v>
       </c>
       <c r="D13" s="2" t="str">
@@ -1449,7 +1450,7 @@
       <c r="B14">
         <v>13</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="6">
         <v>46080.552083333336</v>
       </c>
       <c r="D14" s="2" t="str">
@@ -1472,7 +1473,7 @@
       <c r="B15">
         <v>14</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="6">
         <v>46090.635416666664</v>
       </c>
       <c r="D15" s="2" t="str">
@@ -1495,7 +1496,7 @@
       <c r="B16">
         <v>15</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="6">
         <v>46094.552083333336</v>
       </c>
       <c r="D16" s="2" t="str">
@@ -1518,7 +1519,7 @@
       <c r="B17">
         <v>16</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <v>46097.635416666664</v>
       </c>
       <c r="D17" s="2" t="str">
@@ -1541,7 +1542,7 @@
       <c r="B18">
         <v>17</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="6">
         <v>46101.552083333336</v>
       </c>
       <c r="D18" s="2" t="str">
@@ -1564,7 +1565,7 @@
       <c r="B19">
         <v>18</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="6">
         <v>46104.635416666664</v>
       </c>
       <c r="D19" s="2" t="str">
@@ -1573,11 +1574,11 @@
       </c>
       <c r="E19" s="2" t="str">
         <f>modele!D19</f>
-        <v xml:space="preserve"> </v>
+        <v>Excel</v>
       </c>
       <c r="F19" s="2" t="str">
         <f>modele!E19</f>
-        <v>Formation PowerAutomate</v>
+        <v xml:space="preserve"> </v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1587,7 +1588,7 @@
       <c r="B20">
         <v>19</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <v>46111.635416666664</v>
       </c>
       <c r="D20" s="2" t="str">
@@ -1596,11 +1597,11 @@
       </c>
       <c r="E20" s="2" t="str">
         <f>modele!D20</f>
-        <v xml:space="preserve"> </v>
+        <v>PowerApps</v>
       </c>
       <c r="F20" s="2" t="str">
         <f>modele!E20</f>
-        <v>Simulation de formation (individuel)</v>
+        <v xml:space="preserve"> </v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1610,7 +1611,7 @@
       <c r="B21">
         <v>20</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="6">
         <v>46122.552083333336</v>
       </c>
       <c r="D21" s="2" t="str">
@@ -1619,11 +1620,11 @@
       </c>
       <c r="E21" s="2" t="str">
         <f>modele!D21</f>
-        <v xml:space="preserve"> </v>
+        <v>PowerApps</v>
       </c>
       <c r="F21" s="2" t="str">
         <f>modele!E21</f>
-        <v>Simulation de formation (individuel)</v>
+        <v xml:space="preserve"> </v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1633,7 +1634,7 @@
       <c r="B22">
         <v>21</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="6">
         <v>46125.635416666664</v>
       </c>
       <c r="D22" s="2" t="str">
@@ -1642,11 +1643,11 @@
       </c>
       <c r="E22" s="2" t="str">
         <f>modele!D22</f>
-        <v xml:space="preserve"> </v>
+        <v>Excel</v>
       </c>
       <c r="F22" s="2" t="str">
         <f>modele!E22</f>
-        <v>Simulation de formation (individuel)</v>
+        <v xml:space="preserve"> </v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1656,7 +1657,7 @@
       <c r="B23">
         <v>22</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="6">
         <v>46129.552083333336</v>
       </c>
       <c r="D23" s="2" t="str">
@@ -1679,7 +1680,7 @@
       <c r="B24">
         <v>23</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="6">
         <v>46132.635416666664</v>
       </c>
       <c r="D24" s="2" t="str">
@@ -1688,11 +1689,11 @@
       </c>
       <c r="E24" s="2" t="str">
         <f>modele!D24</f>
-        <v>PowerApps</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="F24" s="2" t="str">
         <f>modele!E24</f>
-        <v xml:space="preserve"> </v>
+        <v>Formation PowerAutomate</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1702,20 +1703,20 @@
       <c r="B25">
         <v>24</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="6">
         <v>46135.552083333336</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="2" t="str">
         <f>modele!C25</f>
-        <v>0</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="E25" s="2" t="str">
         <f>modele!D25</f>
-        <v>PowerApps</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="F25" s="2" t="str">
         <f>modele!E25</f>
-        <v xml:space="preserve"> </v>
+        <v>Simulation de formation (individuel)</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1725,7 +1726,7 @@
       <c r="B26">
         <v>25</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="6">
         <v>46139.635416666664</v>
       </c>
       <c r="D26" s="2" t="str">
@@ -1734,11 +1735,11 @@
       </c>
       <c r="E26" s="2" t="str">
         <f>modele!D26</f>
-        <v>Excel</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="F26" s="2" t="str">
         <f>modele!E26</f>
-        <v xml:space="preserve"> </v>
+        <v>Simulation de formation (individuel)</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1748,7 +1749,7 @@
       <c r="B27">
         <v>26</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="6">
         <v>46140.552083333336</v>
       </c>
       <c r="D27" s="2" t="str">
@@ -1757,11 +1758,11 @@
       </c>
       <c r="E27" s="2" t="str">
         <f>modele!D27</f>
-        <v>Excel</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="F27" s="2" t="str">
         <f>modele!E27</f>
-        <v xml:space="preserve"> </v>
+        <v>Simulation de formation (individuel)</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1771,7 +1772,7 @@
       <c r="B28">
         <v>27</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="6">
         <v>46146.635416666664</v>
       </c>
       <c r="D28" s="2" t="str">
@@ -1794,7 +1795,7 @@
       <c r="B29">
         <v>28</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="6">
         <v>46150.552083333336</v>
       </c>
       <c r="D29" s="2" t="str">
@@ -1817,7 +1818,7 @@
       <c r="B30">
         <v>29</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="6">
         <v>46153.635416666664</v>
       </c>
       <c r="D30" s="2" t="str">
@@ -1840,7 +1841,7 @@
       <c r="B31">
         <v>30</v>
       </c>
-      <c r="C31" s="8">
+      <c r="C31" s="7">
         <v>46157.552083333336</v>
       </c>
       <c r="D31" s="2" t="str">
@@ -1899,7 +1900,7 @@
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>23</v>
       </c>
       <c r="D2" s="2" t="str">
@@ -1922,7 +1923,7 @@
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D3" s="2" t="str">
@@ -1945,7 +1946,7 @@
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="2" t="str">
@@ -1968,7 +1969,7 @@
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>39</v>
       </c>
       <c r="D5" s="2" t="str">
@@ -1991,7 +1992,7 @@
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>25</v>
       </c>
       <c r="D6" s="2" t="str">
@@ -2014,7 +2015,7 @@
       <c r="B7">
         <v>6</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>40</v>
       </c>
       <c r="D7" s="2" t="str">
@@ -2037,7 +2038,7 @@
       <c r="B8">
         <v>7</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D8" s="2" t="str">
@@ -2060,7 +2061,7 @@
       <c r="B9">
         <v>8</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>41</v>
       </c>
       <c r="D9" s="2" t="str">
@@ -2083,7 +2084,7 @@
       <c r="B10">
         <v>9</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="2" t="str">
@@ -2106,7 +2107,7 @@
       <c r="B11">
         <v>10</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D11" s="2" t="str">
@@ -2129,7 +2130,7 @@
       <c r="B12">
         <v>11</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D12" s="2" t="str">
@@ -2152,7 +2153,7 @@
       <c r="B13">
         <v>12</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D13" s="2" t="str">
@@ -2175,7 +2176,7 @@
       <c r="B14">
         <v>13</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="2" t="str">
@@ -2198,7 +2199,7 @@
       <c r="B15">
         <v>14</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D15" s="2" t="str">
@@ -2221,7 +2222,7 @@
       <c r="B16">
         <v>15</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D16" s="2" t="str">
@@ -2244,7 +2245,7 @@
       <c r="B17">
         <v>16</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="2" t="str">
@@ -2267,7 +2268,7 @@
       <c r="B18">
         <v>17</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="4" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="2" t="str">
@@ -2290,19 +2291,19 @@
       <c r="B19">
         <v>18</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D19" s="2" t="str">
         <f>modele!C19</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="E19" s="2" t="str">
-        <f>modele!D19</f>
-        <v xml:space="preserve"> </v>
+      <c r="E19" s="2" t="e">
+        <f>modele!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="F19" s="2" t="str">
-        <f>modele!E19</f>
+        <f>modele!E24</f>
         <v>Formation PowerAutomate</v>
       </c>
     </row>
@@ -2313,19 +2314,19 @@
       <c r="B20">
         <v>19</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="4" t="s">
         <v>32</v>
       </c>
       <c r="D20" s="2" t="str">
         <f>modele!C20</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="E20" s="2" t="str">
-        <f>modele!D20</f>
-        <v xml:space="preserve"> </v>
+      <c r="E20" s="2" t="e">
+        <f>modele!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="F20" s="2" t="str">
-        <f>modele!E20</f>
+        <f>modele!E25</f>
         <v>Simulation de formation (individuel)</v>
       </c>
     </row>
@@ -2336,19 +2337,19 @@
       <c r="B21">
         <v>20</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="4" t="s">
         <v>47</v>
       </c>
       <c r="D21" s="2" t="str">
         <f>modele!C21</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="E21" s="2" t="str">
-        <f>modele!D21</f>
-        <v xml:space="preserve"> </v>
+      <c r="E21" s="2" t="e">
+        <f>modele!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="F21" s="2" t="str">
-        <f>modele!E21</f>
+        <f>modele!E26</f>
         <v>Simulation de formation (individuel)</v>
       </c>
     </row>
@@ -2359,19 +2360,19 @@
       <c r="B22">
         <v>21</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="4" t="s">
         <v>33</v>
       </c>
       <c r="D22" s="2" t="str">
         <f>modele!C22</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="E22" s="2" t="str">
-        <f>modele!D22</f>
-        <v xml:space="preserve"> </v>
+      <c r="E22" s="2" t="e">
+        <f>modele!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="F22" s="2" t="str">
-        <f>modele!E22</f>
+        <f>modele!E27</f>
         <v>Simulation de formation (individuel)</v>
       </c>
     </row>
@@ -2382,7 +2383,7 @@
       <c r="B23">
         <v>22</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="4" t="s">
         <v>48</v>
       </c>
       <c r="D23" s="2" t="str">
@@ -2390,7 +2391,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="E23" s="2" t="str">
-        <f>modele!D23</f>
+        <f>modele!D19</f>
         <v>Excel</v>
       </c>
       <c r="F23" s="2" t="str">
@@ -2405,7 +2406,7 @@
       <c r="B24">
         <v>23</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="4" t="s">
         <v>34</v>
       </c>
       <c r="D24" s="2" t="str">
@@ -2413,12 +2414,12 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="E24" s="2" t="str">
-        <f>modele!D24</f>
+        <f>modele!D20</f>
         <v>PowerApps</v>
       </c>
-      <c r="F24" s="2" t="str">
-        <f>modele!E24</f>
-        <v xml:space="preserve"> </v>
+      <c r="F24" s="2" t="e">
+        <f>modele!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2428,20 +2429,20 @@
       <c r="B25">
         <v>24</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="2" t="str">
         <f>modele!C25</f>
-        <v>0</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="E25" s="2" t="str">
-        <f>modele!D24</f>
+        <f>modele!D20</f>
         <v>PowerApps</v>
       </c>
-      <c r="F25" s="2" t="str">
-        <f>modele!E25</f>
-        <v xml:space="preserve"> </v>
+      <c r="F25" s="2" t="e">
+        <f>modele!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2451,7 +2452,7 @@
       <c r="B26">
         <v>25</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="4" t="s">
         <v>50</v>
       </c>
       <c r="D26" s="2" t="str">
@@ -2459,12 +2460,12 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="E26" s="2" t="str">
-        <f>modele!D25</f>
+        <f>modele!D21</f>
         <v>PowerApps</v>
       </c>
-      <c r="F26" s="2" t="str">
-        <f>modele!E26</f>
-        <v xml:space="preserve"> </v>
+      <c r="F26" s="2" t="e">
+        <f>modele!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2474,7 +2475,7 @@
       <c r="B27">
         <v>26</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D27" s="2" t="str">
@@ -2482,12 +2483,12 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="E27" s="2" t="str">
-        <f>modele!D27</f>
+        <f>modele!D23</f>
         <v>Excel</v>
       </c>
-      <c r="F27" s="2" t="str">
-        <f>modele!E27</f>
-        <v xml:space="preserve"> </v>
+      <c r="F27" s="2" t="e">
+        <f>modele!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2497,7 +2498,7 @@
       <c r="B28">
         <v>27</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="4" t="s">
         <v>51</v>
       </c>
       <c r="D28" s="2" t="str">
@@ -2520,7 +2521,7 @@
       <c r="B29">
         <v>28</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D29" s="2" t="str">
@@ -2543,7 +2544,7 @@
       <c r="B30">
         <v>29</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="4" t="s">
         <v>52</v>
       </c>
       <c r="D30" s="2" t="str">
@@ -2566,7 +2567,7 @@
       <c r="B31">
         <v>30</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="4" t="s">
         <v>37</v>
       </c>
       <c r="D31" s="2" t="str">

</xml_diff>

<commit_message>
ajout horaire de simulation
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/support/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C65A8A18-CE0B-6445-8BDC-E4DC342A8525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381096F6-567C-F048-8D03-B02CDC3DAD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3000" yWindow="1580" windowWidth="27240" windowHeight="16440" activeTab="1" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
+    <workbookView xWindow="3000" yWindow="1580" windowWidth="27240" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
   <sheets>
     <sheet name="modele" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="57">
   <si>
     <t>Date</t>
   </si>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>Comment ajouter un add-on en Word</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</t>
   </si>
 </sst>
 </file>
@@ -989,11 +992,11 @@
       <c r="C23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D23" t="s">
-        <v>16</v>
+      <c r="D23" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -1004,13 +1007,13 @@
         <v>23</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>17</v>
+      <c r="E24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -1021,7 +1024,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>18</v>
@@ -1038,7 +1041,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>18</v>
@@ -1055,7 +1058,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>18</v>
@@ -1666,11 +1669,11 @@
       </c>
       <c r="E23" s="2" t="str">
         <f>modele!D23</f>
-        <v>Excel</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="F23" s="2" t="str">
         <f>modele!E23</f>
-        <v xml:space="preserve"> </v>
+        <v>Formation PowerAutomate</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1685,7 +1688,7 @@
       </c>
       <c r="D24" s="2" t="str">
         <f>modele!C24</f>
-        <v xml:space="preserve"> </v>
+        <v xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</v>
       </c>
       <c r="E24" s="2" t="str">
         <f>modele!D24</f>
@@ -1693,7 +1696,7 @@
       </c>
       <c r="F24" s="2" t="str">
         <f>modele!E24</f>
-        <v>Formation PowerAutomate</v>
+        <v>Simulation de formation (individuel)</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1708,7 +1711,7 @@
       </c>
       <c r="D25" s="2" t="str">
         <f>modele!C25</f>
-        <v xml:space="preserve"> </v>
+        <v xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</v>
       </c>
       <c r="E25" s="2" t="str">
         <f>modele!D25</f>
@@ -1731,7 +1734,7 @@
       </c>
       <c r="D26" s="2" t="str">
         <f>modele!C26</f>
-        <v xml:space="preserve"> </v>
+        <v xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</v>
       </c>
       <c r="E26" s="2" t="str">
         <f>modele!D26</f>
@@ -1754,7 +1757,7 @@
       </c>
       <c r="D27" s="2" t="str">
         <f>modele!C27</f>
-        <v xml:space="preserve"> </v>
+        <v xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</v>
       </c>
       <c r="E27" s="2" t="str">
         <f>modele!D27</f>
@@ -2304,7 +2307,7 @@
       </c>
       <c r="F19" s="2" t="str">
         <f>modele!E24</f>
-        <v>Formation PowerAutomate</v>
+        <v>Simulation de formation (individuel)</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2396,7 +2399,7 @@
       </c>
       <c r="F23" s="2" t="str">
         <f>modele!E23</f>
-        <v xml:space="preserve"> </v>
+        <v>Formation PowerAutomate</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2411,7 +2414,7 @@
       </c>
       <c r="D24" s="2" t="str">
         <f>modele!C24</f>
-        <v xml:space="preserve"> </v>
+        <v xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</v>
       </c>
       <c r="E24" s="2" t="str">
         <f>modele!D20</f>
@@ -2434,7 +2437,7 @@
       </c>
       <c r="D25" s="2" t="str">
         <f>modele!C25</f>
-        <v xml:space="preserve"> </v>
+        <v xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</v>
       </c>
       <c r="E25" s="2" t="str">
         <f>modele!D20</f>
@@ -2457,7 +2460,7 @@
       </c>
       <c r="D26" s="2" t="str">
         <f>modele!C26</f>
-        <v xml:space="preserve"> </v>
+        <v xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</v>
       </c>
       <c r="E26" s="2" t="str">
         <f>modele!D21</f>
@@ -2480,11 +2483,11 @@
       </c>
       <c r="D27" s="2" t="str">
         <f>modele!C27</f>
-        <v xml:space="preserve"> </v>
+        <v xml:space="preserve"> [Horaire de simulation](horaire-eleve.md)</v>
       </c>
       <c r="E27" s="2" t="str">
         <f>modele!D23</f>
-        <v>Excel</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="F27" s="2" t="e">
         <f>modele!#REF!</f>

</xml_diff>

<commit_message>
switch cours 30 mars et 2 avril
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/support/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381096F6-567C-F048-8D03-B02CDC3DAD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8678AE-748A-924C-9091-04FB3D680252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="27240" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -942,7 +942,7 @@
         <v>18</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>18</v>
@@ -976,7 +976,7 @@
         <v>18</v>
       </c>
       <c r="D22" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>18</v>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="E20" s="2" t="str">
         <f>modele!D20</f>
-        <v>PowerApps</v>
+        <v>Excel</v>
       </c>
       <c r="F20" s="2" t="str">
         <f>modele!E20</f>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="E22" s="2" t="str">
         <f>modele!D22</f>
-        <v>Excel</v>
+        <v>PowerApps</v>
       </c>
       <c r="F22" s="2" t="str">
         <f>modele!E22</f>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="E24" s="2" t="str">
         <f>modele!D20</f>
-        <v>PowerApps</v>
+        <v>Excel</v>
       </c>
       <c r="F24" s="2" t="e">
         <f>modele!#REF!</f>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="E25" s="2" t="str">
         <f>modele!D20</f>
-        <v>PowerApps</v>
+        <v>Excel</v>
       </c>
       <c r="F25" s="2" t="e">
         <f>modele!#REF!</f>

</xml_diff>